<commit_message>
Export report tables as CSV for Google Sheets IMPORTDATA
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqykPXBEkntRruusNwAddj
</commit_message>
<xml_diff>
--- a/reports/steady_stack.xlsx
+++ b/reports/steady_stack.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -214,13 +214,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -244,7 +244,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -285,8 +285,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -309,13 +309,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -338,14 +338,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -386,8 +386,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -410,13 +410,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -439,14 +439,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -489,8 +489,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -513,13 +513,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -542,14 +542,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -575,14 +575,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -624,8 +624,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -651,7 +651,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -666,9 +666,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -688,9 +688,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -700,7 +700,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -715,9 +715,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -737,9 +737,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1054,7 +1054,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>อัปเดตอัตโนมัติ 2026-10-21 21:23 (เวลาไทย) · ตัวเลขเป็นบาท</t>
+          <t>อัปเดตอัตโนมัติ 2026-10-21 21:45 (เวลาไทย) · ตัวเลขเป็นบาท</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>-0.009523846153846155</v>
+        <v>-0.009523846153846154</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Report: historical capital = money put into bot, so profit-vs-capital chart is continuous
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqykPXBEkntRruusNwAddj
</commit_message>
<xml_diff>
--- a/reports/steady_stack.xlsx
+++ b/reports/steady_stack.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -214,13 +214,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -244,7 +244,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -285,8 +285,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -309,13 +309,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -338,14 +338,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -386,8 +386,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -410,13 +410,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -439,14 +439,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -489,8 +489,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -513,13 +513,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -542,14 +542,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -575,14 +575,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -624,8 +624,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -651,7 +651,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -666,9 +666,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -688,9 +688,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -700,7 +700,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -715,9 +715,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -737,9 +737,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1054,7 +1054,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>อัปเดตอัตโนมัติ 2026-10-21 22:20 (เวลาไทย) · ตัวเลขเป็นบาท</t>
+          <t>อัปเดตอัตโนมัติ 2026-10-21 23:09 (เวลาไทย) · ตัวเลขเป็นบาท</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>-0.009523846153846155</v>
+        <v>-0.009523846153846154</v>
       </c>
     </row>
     <row r="17">
@@ -5823,7 +5823,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ก่อนเริ่มโหมดทั้งบัญชี = เฉพาะเงินของบอท (ทุน 700) · หลังจากนั้น = ทั้งบัญชี (มูลค่ากระโดดตอนเปลี่ยนโหมด ไม่ใช่กำไร — ดูกราฟกำไรเทียบทุนแทน)</t>
+          <t>ก่อนเริ่มโหมดทั้งบัญชี = เฉพาะเงินของบอท (ทุน = เงินที่เติมเข้าบอท) · หลังจากนั้น = ทั้งบัญชี (มูลค่ากระโดดตอนเปลี่ยนโหมด ไม่ใช่กำไร — ดูกราฟกำไรเทียบทุนแทน)</t>
         </is>
       </c>
     </row>
@@ -5877,10 +5877,10 @@
         <v>399.9</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>-300.1</v>
+        <v>-0.1</v>
       </c>
       <c r="E4" s="12" t="n">
         <v>399.9</v>
@@ -5903,10 +5903,10 @@
         <v>399.1</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>-300.9</v>
+        <v>-0.9</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>399.1</v>
@@ -5929,10 +5929,10 @@
         <v>399.04</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>-300.96</v>
+        <v>-0.96</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>399.04</v>
@@ -5955,10 +5955,10 @@
         <v>399.25</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>-300.75</v>
+        <v>-0.75</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>399.25</v>

</xml_diff>

<commit_message>
Dip-buying reserve pool: 30% of capital, buy -10% from 72h high, TP +6% / SL -20%, funded from sale proceeds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqykPXBEkntRruusNwAddj
</commit_message>
<xml_diff>
--- a/reports/steady_stack.xlsx
+++ b/reports/steady_stack.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -214,13 +214,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -244,7 +244,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -285,8 +285,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -309,13 +309,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -338,14 +338,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -386,8 +386,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -410,13 +410,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -439,14 +439,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -489,8 +489,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -513,13 +513,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -542,14 +542,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -575,14 +575,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -624,8 +624,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -651,7 +651,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -666,9 +666,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -688,9 +688,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -700,7 +700,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -715,9 +715,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -737,9 +737,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1054,7 +1054,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>อัปเดตอัตโนมัติ 2026-10-22 22:23 (เวลาไทย) · ตัวเลขเป็นบาท</t>
+          <t>อัปเดตอัตโนมัติ 2026-10-22 22:37 (เวลาไทย) · ตัวเลขเป็นบาท</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>-0.009523846153846155</v>
+        <v>-0.009523846153846154</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Weekly strategy tuner: shadow-test bounded params vs live, auto-promote after 3 straight weekly wins; bot loads clamped tuned params; report/dashboard show tuner status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqykPXBEkntRruusNwAddj
</commit_message>
<xml_diff>
--- a/reports/steady_stack.xlsx
+++ b/reports/steady_stack.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="พอร์ตตอนนี้" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ระบบตัดสินใจ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติซื้อ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ประวัติขาย" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="กำไรขาดทุน" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="มูลค่าพอร์ต" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="เหตุการณ์" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -214,13 +214,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -244,7 +244,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -285,8 +285,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -309,13 +309,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -338,14 +338,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -386,8 +386,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -410,13 +410,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -439,14 +439,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -489,8 +489,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -513,13 +513,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -542,14 +542,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -575,14 +575,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -624,8 +624,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -651,7 +651,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -666,9 +666,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -688,9 +688,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -700,7 +700,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -715,9 +715,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -737,9 +737,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1054,7 +1054,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>อัปเดตอัตโนมัติ 2026-10-28 10:28 (เวลาไทย) · ตัวเลขเป็นบาท</t>
+          <t>อัปเดตอัตโนมัติ 2026-10-28 10:51 (เวลาไทย) · ตัวเลขเป็นบาท</t>
         </is>
       </c>
     </row>

</xml_diff>